<commit_message>
update to neyman interval code
</commit_message>
<xml_diff>
--- a/primary_genes/top9_95CI_primary.xlsx
+++ b/primary_genes/top9_95CI_primary.xlsx
@@ -1,68 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10916"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anqiwang/Documents/GitHub/Ozone-and-Lung-Functions/primary genes/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDD4CBBE-1C7C-4C42-9411-E5C21FB538AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12840" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
-  <si>
-    <t>CpG</t>
-  </si>
-  <si>
-    <t>lower_bound</t>
-  </si>
-  <si>
-    <t>upper_bound</t>
-  </si>
-  <si>
-    <t>cg03610073</t>
-  </si>
-  <si>
-    <t>cg18652319</t>
-  </si>
-  <si>
-    <t>cg03995486</t>
-  </si>
-  <si>
-    <t>cg01133890</t>
-  </si>
-  <si>
-    <t>cg05106269</t>
-  </si>
-  <si>
-    <t>cg00087425</t>
-  </si>
-  <si>
-    <t>cg02680732</t>
-  </si>
-  <si>
-    <t>cg16547110</t>
-  </si>
-  <si>
-    <t>cg10950028</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -110,21 +63,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -162,7 +107,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -196,7 +141,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -231,10 +175,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -407,123 +350,142 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="14.5" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>3</v>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CpG</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>lower_bound</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>upper_bound</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>cg03610073</t>
+        </is>
       </c>
       <c r="B2">
-        <v>-2.9489066208019801E-2</v>
+        <v>-0.0294890662080198</v>
       </c>
       <c r="C2">
-        <v>-7.9140101204990092E-3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>4</v>
+        <v>-0.007914010120499009</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>cg18652319</t>
+        </is>
       </c>
       <c r="B3">
-        <v>4.6566565481282401E-4</v>
+        <v>0.000465665654812824</v>
       </c>
       <c r="C3">
-        <v>4.4589013287096397E-3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>5</v>
+        <v>0.00445890132870964</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cg03995486</t>
+        </is>
       </c>
       <c r="B4">
-        <v>1.4876198154931599E-3</v>
+        <v>0.00148761981549316</v>
       </c>
       <c r="C4">
-        <v>1.5644116397419802E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>6</v>
+        <v>0.0156441163974198</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>cg01133890</t>
+        </is>
       </c>
       <c r="B5">
-        <v>-2.08822037966458E-2</v>
+        <v>-0.0208822037966458</v>
       </c>
       <c r="C5">
-        <v>-2.1620653632704501E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>7</v>
+        <v>-0.00216206536327046</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>cg05106269</t>
+        </is>
       </c>
       <c r="B6">
-        <v>6.2308692818294003E-4</v>
+        <v>0.00062308692818294</v>
       </c>
       <c r="C6">
-        <v>1.90855794104513E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>8</v>
+        <v>0.0190855794104513</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>cg00087425</t>
+        </is>
       </c>
       <c r="B7">
-        <v>2.3171647372814898E-3</v>
+        <v>0.0023171647372815</v>
       </c>
       <c r="C7">
-        <v>4.4288841979833203E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>9</v>
+        <v>0.0442888419798332</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>cg02680732</t>
+        </is>
       </c>
       <c r="B8">
-        <v>-6.7223176270956699E-3</v>
+        <v>-0.00672231762709567</v>
       </c>
       <c r="C8">
-        <v>-1.5006696589573199E-4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>10</v>
+        <v>-0.000150066965895732</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>cg16547110</t>
+        </is>
       </c>
       <c r="B9">
-        <v>2.20423763105907E-4</v>
+        <v>0.000220423763105907</v>
       </c>
       <c r="C9">
-        <v>1.02641162587917E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>11</v>
+        <v>0.0102641162587917</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>cg10950028</t>
+        </is>
       </c>
       <c r="B10">
-        <v>-3.2103027542245498E-2</v>
+        <v>-0.0321030275422455</v>
       </c>
       <c r="C10">
-        <v>6.3764656606576898E-4</v>
+        <v>0.000637646566065769</v>
       </c>
     </row>
   </sheetData>

</xml_diff>